<commit_message>
Daily NSE scan: 2026-09-10
</commit_message>
<xml_diff>
--- a/output/2026-09-10/enriched_analysis.xlsx
+++ b/output/2026-09-10/enriched_analysis.xlsx
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.43</v>
+        <v>0.429</v>
       </c>
       <c r="Q3" t="n">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="R3" t="n">
-        <v>26.2</v>
+        <v>26.3</v>
       </c>
       <c r="S3" t="n">
         <v>19</v>
@@ -1177,10 +1177,10 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>3.621</v>
+        <v>3.622</v>
       </c>
       <c r="Q4" t="n">
-        <v>2925</v>
+        <v>2924</v>
       </c>
       <c r="R4" t="n">
         <v>22.9</v>
@@ -1362,10 +1362,10 @@
         <v>0.062</v>
       </c>
       <c r="Q5" t="n">
-        <v>1323</v>
+        <v>1327</v>
       </c>
       <c r="R5" t="n">
-        <v>17.8</v>
+        <v>17.9</v>
       </c>
       <c r="S5" t="n">
         <v>55</v>
@@ -1521,33 +1521,33 @@
         <v>71.12</v>
       </c>
       <c r="J6" t="n">
-        <v>70.48999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
         <v>72.56999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>1.32</v>
+        <v>1.52</v>
       </c>
       <c r="N6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.638</v>
+        <v>0.738</v>
       </c>
       <c r="Q6" t="n">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="R6" t="n">
-        <v>8.81</v>
+        <v>8.75</v>
       </c>
       <c r="S6" t="n">
         <v>17</v>
@@ -1583,10 +1583,10 @@
         <v>60</v>
       </c>
       <c r="AD6" t="n">
-        <v>70.48752536580156</v>
+        <v>70.40347079627149</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
@@ -1610,53 +1610,53 @@
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AL6" t="n">
         <v>24</v>
       </c>
       <c r="AM6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AN6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AO6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AP6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AQ6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AR6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AS6" t="n">
-        <v>2797000</v>
+        <v>4786562</v>
       </c>
       <c r="AT6" t="n">
-        <v>5480343</v>
+        <v>7469905</v>
       </c>
       <c r="AU6" t="n">
-        <v>13199494</v>
+        <v>15189056</v>
       </c>
       <c r="AV6" t="n">
-        <v>13199494</v>
+        <v>15189056</v>
       </c>
       <c r="AW6" t="n">
-        <v>13199494</v>
+        <v>15189056</v>
       </c>
       <c r="AX6" t="n">
-        <v>2797000</v>
+        <v>4786562</v>
       </c>
       <c r="AY6" t="n">
-        <v>13199494</v>
+        <v>15189056</v>
       </c>
       <c r="AZ6" t="n">
         <v>1</v>
@@ -1665,7 +1665,7 @@
         <v>0</v>
       </c>
       <c r="BB6" t="n">
-        <v>0.2119</v>
+        <v>0.3151</v>
       </c>
     </row>
     <row r="7">
@@ -1726,10 +1726,10 @@
         <v>0.048</v>
       </c>
       <c r="Q7" t="n">
-        <v>16100</v>
+        <v>16040</v>
       </c>
       <c r="R7" t="n">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="S7" t="n">
         <v>16</v>
@@ -1908,10 +1908,10 @@
         <v>0.145</v>
       </c>
       <c r="Q8" t="n">
-        <v>2160</v>
+        <v>2165</v>
       </c>
       <c r="R8" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="S8" t="n">
         <v>-3</v>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.309</v>
+        <v>0.31</v>
       </c>
       <c r="Q9" t="n">
-        <v>2752</v>
+        <v>2736</v>
       </c>
       <c r="R9" t="n">
-        <v>22.5</v>
+        <v>22.4</v>
       </c>
       <c r="S9" t="n">
         <v>8</v>
@@ -2449,13 +2449,13 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.045</v>
+        <v>0.046</v>
       </c>
       <c r="Q11" t="n">
-        <v>15860</v>
+        <v>15805</v>
       </c>
       <c r="R11" t="n">
-        <v>40.4</v>
+        <v>40.2</v>
       </c>
       <c r="S11" t="n">
         <v>83</v>
@@ -2631,13 +2631,13 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.075</v>
+        <v>0.076</v>
       </c>
       <c r="Q12" t="n">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="R12" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="S12" t="n">
         <v>-8</v>
@@ -3177,13 +3177,13 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.136</v>
+        <v>0.135</v>
       </c>
       <c r="Q15" t="n">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="R15" t="n">
-        <v>5.95</v>
+        <v>5.97</v>
       </c>
       <c r="S15" t="n">
         <v>118</v>
@@ -3374,7 +3374,7 @@
         <v>31.98</v>
       </c>
       <c r="W16" t="n">
-        <v>0.27</v>
+        <v>-0.26</v>
       </c>
       <c r="X16" t="n">
         <v>0.1</v>
@@ -3535,13 +3535,13 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="Q17" t="n">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="R17" t="n">
-        <v>32.7</v>
+        <v>32.5</v>
       </c>
       <c r="S17" t="n">
         <v>24</v>
@@ -3559,7 +3559,7 @@
         <v>4.96</v>
       </c>
       <c r="X17" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Y17" t="b">
         <v>1</v>
@@ -3720,10 +3720,10 @@
         <v>0.178</v>
       </c>
       <c r="Q18" t="n">
-        <v>1693</v>
+        <v>1688</v>
       </c>
       <c r="R18" t="n">
-        <v>59</v>
+        <v>58.9</v>
       </c>
       <c r="S18" t="n">
         <v>7</v>
@@ -4445,13 +4445,13 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>0.452</v>
+        <v>0.455</v>
       </c>
       <c r="Q22" t="n">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="R22" t="n">
-        <v>1301</v>
+        <v>1291</v>
       </c>
       <c r="S22" t="n">
         <v>-61</v>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -5349,13 +5349,13 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.171</v>
+        <v>0.172</v>
       </c>
       <c r="Q27" t="n">
-        <v>903</v>
+        <v>893</v>
       </c>
       <c r="R27" t="n">
-        <v>8.880000000000001</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="S27" t="n">
         <v>7</v>
@@ -5895,10 +5895,10 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.391</v>
+        <v>0.392</v>
       </c>
       <c r="Q30" t="n">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="R30" t="n">
         <v>105</v>
@@ -6283,7 +6283,7 @@
         <v>1.58</v>
       </c>
       <c r="X32" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Y32" t="b">
         <v>0</v>
@@ -6444,7 +6444,7 @@
         <v>0.051</v>
       </c>
       <c r="Q33" t="n">
-        <v>5182</v>
+        <v>5186</v>
       </c>
       <c r="R33" t="n">
         <v>33.8</v>
@@ -6805,13 +6805,13 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.948</v>
+        <v>0.95</v>
       </c>
       <c r="Q35" t="n">
-        <v>5105</v>
+        <v>5093</v>
       </c>
       <c r="R35" t="n">
-        <v>40.9</v>
+        <v>40.8</v>
       </c>
       <c r="S35" t="n">
         <v>0</v>
@@ -7352,7 +7352,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="Q38" t="n">
-        <v>53935</v>
+        <v>53987</v>
       </c>
       <c r="R38" t="n">
         <v>45.7</v>
@@ -7531,13 +7531,13 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.189</v>
+        <v>0.187</v>
       </c>
       <c r="Q39" t="n">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="R39" t="n">
-        <v>23.6</v>
+        <v>24</v>
       </c>
       <c r="S39" t="n">
         <v>12</v>
@@ -7713,13 +7713,13 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.505</v>
+        <v>0.5</v>
       </c>
       <c r="Q40" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="R40" t="n">
-        <v>74.3</v>
+        <v>74.8</v>
       </c>
       <c r="S40" t="n">
         <v>-1</v>
@@ -7898,10 +7898,10 @@
         <v>0.002</v>
       </c>
       <c r="Q41" t="n">
-        <v>325632</v>
+        <v>328407</v>
       </c>
       <c r="R41" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="S41" t="n">
         <v>7</v>
@@ -8978,7 +8978,7 @@
         <v>0.6</v>
       </c>
       <c r="Q47" t="n">
-        <v>1813</v>
+        <v>1812</v>
       </c>
       <c r="R47" t="n">
         <v>32.7</v>
@@ -9875,23 +9875,23 @@
         <v>71.12</v>
       </c>
       <c r="D6" t="n">
-        <v>70.48999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>72.56999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>1.32</v>
+        <v>1.52</v>
       </c>
       <c r="H6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
     </row>
@@ -10463,7 +10463,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C23" t="n">

</xml_diff>